<commit_message>
Cerrar resultados finales del día
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -666,6 +666,908 @@
         </is>
       </c>
       <c r="I6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Southend vs Cambridge United</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Southend</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Muras United vs Bars</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Muras United</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Spartak Trnava vs Beşiktaş</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Beşiktaş</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F9" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Eintracht Braunschweig vs Havelse</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Havelse</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F10" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Levski Sofia vs Borac Banja Luka</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Levski Sofia</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F11" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Grotta vs Grindavik</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Grindavik</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F12" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bristol Rovers vs Leicester</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bristol Rovers</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F13" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Woking vs Portsmouth</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Woking</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F14" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Dover vs Gillingham</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dover</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F15" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Keith vs Aberdeen U21</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Keith</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="F16" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sutton Athletic vs Dartford</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sutton Athletic</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F17" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Evesham United vs Worcester City</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Evesham United</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F18" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Annan Athletic vs Dundee</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Annan Athletic</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F19" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Brechin vs Livingston</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Brechin</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F20" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Brora Rangers vs Aberdeen</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Brora Rangers</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F21" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Clyde vs Airdrie United</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Clyde</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F22" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Elgin City vs Peterhead</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Elgin City</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F23" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Forfar Athletic vs Partick</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Forfar Athletic</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F24" t="n">
+        <v>88</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bath City vs Cardiff City U21</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Bath City</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F25" t="n">
+        <v>88</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cork City vs Cardiff</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Cardiff</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F26" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Larne vs Tre Fiori</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Larne</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F27" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Shamrock Rovers vs Floriana</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Shamrock Rovers</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F28" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -680,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -737,6 +1639,25 @@
         <v>93</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>22</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>